<commit_message>
fix(pytools): bound used-range summary batch memory
</commit_message>
<xml_diff>
--- a/pytools-core/tests/fixtures/summary_used_range/error_value.xlsx
+++ b/pytools-core/tests/fixtures/summary_used_range/error_value.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ErrorCase" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +413,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="e">
         <v>#DIV/0!</v>
       </c>
+      <c r="B1" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="C1" t="e">
+        <v>#NAME?</v>
+      </c>
+      <c r="D1" t="e">
+        <v>#NULL!</v>
+      </c>
+      <c r="E1" t="e">
+        <v>#NUM!</v>
+      </c>
+      <c r="F1" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="G1" t="e">
+        <v>#VALUE!</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
test(pytools): cover empty and unsupported summary errors
</commit_message>
<xml_diff>
--- a/pytools-core/tests/fixtures/summary_used_range/error_value.xlsx
+++ b/pytools-core/tests/fixtures/summary_used_range/error_value.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empty" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,4 +443,17 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>